<commit_message>
minor changes in excel and middleware added
</commit_message>
<xml_diff>
--- a/public/file/Trax Bulk City Add.xlsx
+++ b/public/file/Trax Bulk City Add.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Trax\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sonic\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FACBF5-562B-4FA3-BF74-D96D31785D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48C450C-AAEA-4FA1-A107-739EE391961B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>select_hub</t>
   </si>
@@ -103,18 +103,6 @@
     <t>reverse_pickup_same_day</t>
   </si>
   <si>
-    <t>ptl_rush</t>
-  </si>
-  <si>
-    <t>ptl_saver_plus</t>
-  </si>
-  <si>
-    <t>ptl_swift</t>
-  </si>
-  <si>
-    <t>ptl_same_day</t>
-  </si>
-  <si>
     <t>walkin_rush</t>
   </si>
   <si>
@@ -124,18 +112,12 @@
     <t>walkin_swift</t>
   </si>
   <si>
-    <t>walkin_same_day</t>
-  </si>
-  <si>
     <t>City Name</t>
   </si>
   <si>
     <t>City Code</t>
   </si>
   <si>
-    <t>AHMAD</t>
-  </si>
-  <si>
     <t>is_city</t>
   </si>
   <si>
@@ -166,35 +148,29 @@
     <t>osa_rate_4</t>
   </si>
   <si>
-    <t>Ahmad</t>
-  </si>
-  <si>
-    <t>Hasan</t>
-  </si>
-  <si>
     <t>closest_hub</t>
   </si>
   <si>
     <t>vehicle_list</t>
   </si>
   <si>
-    <t>Fresh 2</t>
-  </si>
-  <si>
-    <t>Fresh 3</t>
-  </si>
-  <si>
-    <t>Fresh 4</t>
-  </si>
-  <si>
-    <t>ds</t>
+    <t>ftl_same_day</t>
+  </si>
+  <si>
+    <t>ftl_saver_plus</t>
+  </si>
+  <si>
+    <t>ftl_swift</t>
+  </si>
+  <si>
+    <t>ftl_rush</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,14 +182,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -268,25 +236,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -589,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AW8"/>
+  <dimension ref="A1:AV8"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -606,29 +571,33 @@
     <col min="12" max="13" width="20.77734375" customWidth="1"/>
     <col min="14" max="14" width="25.109375" customWidth="1"/>
     <col min="15" max="15" width="15.44140625" customWidth="1"/>
-    <col min="40" max="40" width="19.33203125" customWidth="1"/>
-    <col min="41" max="41" width="23.33203125" customWidth="1"/>
-    <col min="42" max="42" width="17.44140625" customWidth="1"/>
-    <col min="43" max="43" width="18.6640625" customWidth="1"/>
-    <col min="44" max="44" width="21.21875" customWidth="1"/>
-    <col min="45" max="45" width="20" customWidth="1"/>
-    <col min="46" max="46" width="21.5546875" customWidth="1"/>
-    <col min="47" max="47" width="23.109375" customWidth="1"/>
-    <col min="48" max="49" width="19.109375" customWidth="1"/>
+    <col min="32" max="32" width="30.77734375" customWidth="1"/>
+    <col min="33" max="33" width="21.21875" customWidth="1"/>
+    <col min="34" max="34" width="16.44140625" customWidth="1"/>
+    <col min="35" max="35" width="20.33203125" customWidth="1"/>
+    <col min="39" max="39" width="19.33203125" customWidth="1"/>
+    <col min="40" max="40" width="23.33203125" customWidth="1"/>
+    <col min="41" max="41" width="17.44140625" customWidth="1"/>
+    <col min="42" max="42" width="18.6640625" customWidth="1"/>
+    <col min="43" max="43" width="21.21875" customWidth="1"/>
+    <col min="44" max="44" width="20" customWidth="1"/>
+    <col min="45" max="45" width="21.5546875" customWidth="1"/>
+    <col min="46" max="46" width="23.109375" customWidth="1"/>
+    <col min="47" max="48" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49">
+    <row r="1" spans="1:48">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
@@ -712,198 +681,59 @@
         <v>26</v>
       </c>
       <c r="AF1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="AM1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="AN1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AR1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AU1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AQ1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AV1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AV1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AW1" s="3" t="s">
-        <v>51</v>
-      </c>
     </row>
-    <row r="2" spans="1:49">
-      <c r="A2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>202</v>
-      </c>
-      <c r="G2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H2">
-        <v>10</v>
-      </c>
-      <c r="I2">
-        <v>10</v>
-      </c>
-      <c r="J2">
-        <v>10</v>
-      </c>
-      <c r="K2">
-        <v>10</v>
-      </c>
-      <c r="L2">
-        <v>10</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO2">
-        <v>1</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>49</v>
-      </c>
-      <c r="AQ2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:49">
-      <c r="A3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>202</v>
-      </c>
-      <c r="H3">
-        <v>10</v>
-      </c>
-      <c r="I3">
-        <v>10</v>
-      </c>
-      <c r="J3">
-        <v>10</v>
-      </c>
-      <c r="K3">
-        <v>10</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>1</v>
-      </c>
-      <c r="AN3" s="2"/>
-    </row>
-    <row r="4" spans="1:49">
-      <c r="A4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4">
-        <v>20</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>202</v>
-      </c>
-      <c r="G4" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4">
-        <v>10</v>
-      </c>
-      <c r="I4">
-        <v>10</v>
-      </c>
-      <c r="J4">
-        <v>10</v>
-      </c>
-      <c r="K4">
-        <v>10</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>1</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>55</v>
-      </c>
-      <c r="AO4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:49">
-      <c r="AV8" s="4"/>
+    <row r="8" spans="1:48">
+      <c r="AU8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>